<commit_message>
Improved folder structure. Minor code adjustments.
</commit_message>
<xml_diff>
--- a/pipeline/first_level_analysis/contrasts.xlsx
+++ b/pipeline/first_level_analysis/contrasts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thesis-matlab-pipeline\analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thesis-matlab-pipeline\pipeline\first_level_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB34203F-5603-426C-BA6B-AD9170CFCF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A5FC09B-D204-49CF-8872-17755B59990D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -613,5 +613,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Changes on MCF conversion script: Cue as nuisance regressor included; compatibility for old and new log format. Old conversion script removed. Improvements on preprocessing and first-level pipeline.
</commit_message>
<xml_diff>
--- a/pipeline/first_level_analysis/contrasts.xlsx
+++ b/pipeline/first_level_analysis/contrasts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thesis-matlab-pipeline\pipeline\first_level_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A5FC09B-D204-49CF-8872-17755B59990D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E877BEC4-DBC4-4B4B-A186-2841C84BCCC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7275" yWindow="2475" windowWidth="14490" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="25">
   <si>
     <t>Contrast</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>0 -1 1 0 0 0 0 0 0 0 0</t>
+  </si>
+  <si>
+    <t>incongruent_real &lt; incongruent_fake</t>
   </si>
 </sst>
 </file>
@@ -596,7 +599,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
         <v>23</v>

</xml_diff>